<commit_message>
Apply final review fixes: facts, mobile layout, GCB styling, data files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/2025/LowLatencyGCB_2025_v1.0.xlsx
+++ b/downloads/2025/LowLatencyGCB_2025_v1.0.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -548,107 +548,131 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Citation</t>
+          <t>Atmospheric growth</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Manuscript in review — Low latency global carbon budget reveals strong land sink recovery in 2025</t>
+          <t>NOAA_MBL: NOAA globally averaged marine boundary layer; MaunaLoa: NOAA Mauna Loa; GRESO: satellite-derived growth rate (GOSAT before 2015, mean of OCO-2 and GOSAT from 2015); OCO2_inversions: mean growth rate implied by the OCO-2 inversions</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Licence</t>
+          <t>Monthly growth &amp; ENSO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution 4.0 International (CC BY 4.0)</t>
+          <t>oni_degC: Oceanic Niño Index (NOAA); GISTEMP: global surface temperature anomaly (NASA GISTEMP)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Citation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Manuscript in review — Low latency global carbon budget reveals strong land sink recovery in 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Licence</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Creative Commons Attribution 4.0 International (CC BY 4.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Contact</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Philippe Ciais &lt;philippe.ciais@cea.fr&gt;; Piyu Ke &lt;piyu.ke@lsce.ipsl.fr&gt;</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Contents</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Global budget</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Annual global CO2 budget, bottom-up and top-down</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Atmospheric growth</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Annual atmospheric CO2 growth rate (ppm yr-1)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Monthly growth &amp; ENSO</t>
+          <t>Global budget</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Monthly CO2 growth rate, ONI and GISTEMP anomaly</t>
+          <t>Annual global CO2 budget, bottom-up and top-down</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Inversions by member</t>
+          <t>Atmospheric growth</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Net land sink from each OCO-2 inversion (GtC yr-1)</t>
+          <t>Annual atmospheric CO2 growth rate (ppm yr-1)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Monthly growth &amp; ENSO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Monthly CO2 growth rate, ONI and GISTEMP anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Inversions by member</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Net land sink from each OCO-2 inversion (GtC yr-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Recovery statistics</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>2025 recovery of the 2023-2024 land-sink loss by region</t>
         </is>
@@ -669,29 +693,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="31" customWidth="1" min="11" max="11"/>
-    <col width="33" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="33" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="23" customWidth="1" min="18" max="18"/>
-    <col width="25" customWidth="1" min="19" max="19"/>
-    <col width="28" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="21" customWidth="1" min="23" max="23"/>
-    <col width="27" customWidth="1" min="24" max="24"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="41" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="27" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="32" customWidth="1" min="19" max="19"/>
+    <col width="35" customWidth="1" min="20" max="20"/>
+    <col width="27" customWidth="1" min="21" max="21"/>
+    <col width="33" customWidth="1" min="22" max="22"/>
+    <col width="28" customWidth="1" min="23" max="23"/>
+    <col width="34" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -702,117 +726,117 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>fossil_emissions</t>
+          <t>fossil_emissions_GtC_yr</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>atmospheric_growth_ppm</t>
+          <t>atmospheric_growth_ppm_GtC_yr</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>atmospheric_growth_ppm_unc</t>
+          <t>atmospheric_growth_ppm_unc_GtC_yr</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>atmospheric_growth_GtC</t>
+          <t>atmospheric_growth_GtC_yr</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ocean_sink_bottom_up</t>
+          <t>ocean_sink_bottom_up_GtC_yr</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ocean_sink_bottom_up_sd</t>
+          <t>ocean_sink_bottom_up_sd_GtC_yr</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>land_sink_bottom_up</t>
+          <t>land_sink_bottom_up_GtC_yr</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>land_sink_bottom_up_sd</t>
+          <t>land_sink_bottom_up_sd_GtC_yr</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>budget_imbalance_bottom_up</t>
+          <t>budget_imbalance_bottom_up_GtC_yr</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>budget_imbalance_bottom_up_sd</t>
+          <t>budget_imbalance_bottom_up_sd_GtC_yr</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>budget_imbalance_bottom_up_p2.5</t>
+          <t>budget_imbalance_bottom_up_p2.5_GtC_yr</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>budget_imbalance_bottom_up_p97.5</t>
+          <t>budget_imbalance_bottom_up_p97.5_GtC_yr</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>atmospheric_growth_GtC_top_down</t>
+          <t>atmospheric_growth_top_down_GtC_yr</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>ocean_sink_top_down</t>
+          <t>ocean_sink_top_down_GtC_yr</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>ocean_sink_top_down_sd</t>
+          <t>ocean_sink_top_down_sd_GtC_yr</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>land_sink_top_down</t>
+          <t>land_sink_top_down_GtC_yr</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>land_sink_top_down_sd</t>
+          <t>land_sink_top_down_sd_GtC_yr</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>budget_closure_top_down</t>
+          <t>budget_closure_top_down_GtC_yr</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>budget_closure_top_down_sd</t>
+          <t>budget_closure_top_down_sd_GtC_yr</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>land_sink_combined</t>
+          <t>land_sink_combined_GtC_yr</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>land_sink_combined_sigma</t>
+          <t>land_sink_combined_sigma_GtC_yr</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>ocean_sink_combined</t>
+          <t>ocean_sink_combined_GtC_yr</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>ocean_sink_combined_sigma</t>
+          <t>ocean_sink_combined_sigma_GtC_yr</t>
         </is>
       </c>
     </row>
@@ -1885,12 +1909,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1901,32 +1925,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>mbl</t>
+          <t>NOAA_MBL_growth_ppm_yr</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>mbl_unc</t>
+          <t>NOAA_MBL_growth_unc_ppm_yr</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>mlo</t>
+          <t>MaunaLoa_growth_ppm_yr</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>mlo_unc</t>
+          <t>MaunaLoa_growth_unc_ppm_yr</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>greso</t>
+          <t>GRESO_growth_ppm_yr</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>oco2_inversions</t>
+          <t>OCO2_inversions_growth_ppm_yr</t>
         </is>
       </c>
     </row>

</xml_diff>